<commit_message>
main Cal main Data Extract and main Val changed to capture non linearity, two linear curves for calibration for all Qs, not yet considering Q affects low slope part
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="22" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="47" uniqueCount="13">
   <si>
     <t>Q</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>RMSE</t>
+  </si>
+  <si>
+    <t>nlCoef</t>
+  </si>
+  <si>
+    <t>n2</t>
   </si>
 </sst>
 </file>
@@ -91,7 +97,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="true"/>
@@ -99,7 +105,9 @@
     <col min="3" max="3" width="12.5546875" customWidth="true"/>
     <col min="4" max="4" width="11.5546875" customWidth="true"/>
     <col min="5" max="5" width="11.5546875" customWidth="true"/>
-    <col min="6" max="6" width="11.5546875" customWidth="true"/>
+    <col min="6" max="6" width="12.5546875" customWidth="true"/>
+    <col min="7" max="7" width="12.21875" customWidth="true"/>
+    <col min="8" max="8" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -119,6 +127,12 @@
         <v>9</v>
       </c>
       <c r="F1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="0" t="s">
         <v>10</v>
       </c>
     </row>
@@ -139,6 +153,12 @@
         <v>203.80348777036431</v>
       </c>
       <c r="F2" s="0">
+        <v>0.11855530366764189</v>
+      </c>
+      <c r="G2" s="0">
+        <v>-24.16198438114008</v>
+      </c>
+      <c r="H2" s="0">
         <v>3.370244958964272</v>
       </c>
     </row>
@@ -159,6 +179,12 @@
         <v>167.52600323946646</v>
       </c>
       <c r="F3" s="0">
+        <v>0.13213001406649094</v>
+      </c>
+      <c r="G3" s="0">
+        <v>-22.13521316453371</v>
+      </c>
+      <c r="H3" s="0">
         <v>1.7850791804303163</v>
       </c>
     </row>
@@ -179,6 +205,12 @@
         <v>151.29005830812935</v>
       </c>
       <c r="F4" s="0">
+        <v>0.16396348347376799</v>
+      </c>
+      <c r="G4" s="0">
+        <v>-24.80604497515036</v>
+      </c>
+      <c r="H4" s="0">
         <v>2.3111601242641355</v>
       </c>
     </row>
@@ -199,6 +231,12 @@
         <v>155.71388203007447</v>
       </c>
       <c r="F5" s="0">
+        <v>0.19859162763641647</v>
+      </c>
+      <c r="G5" s="0">
+        <v>-30.923473277937433</v>
+      </c>
+      <c r="H5" s="0">
         <v>2.4658007191273112</v>
       </c>
     </row>
@@ -219,6 +257,12 @@
         <v>164.69628953709582</v>
       </c>
       <c r="F6" s="0">
+        <v>0.15960913435486068</v>
+      </c>
+      <c r="G6" s="0">
+        <v>-26.287032204473363</v>
+      </c>
+      <c r="H6" s="0">
         <v>3.3545980071603134</v>
       </c>
     </row>

</xml_diff>

<commit_message>
no Q effect considered, back to old version
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="203" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="216" uniqueCount="14">
   <si>
     <t>Q</t>
   </si>
@@ -106,9 +106,9 @@
     <col min="1" max="1" width="4.5703125" customWidth="true"/>
     <col min="2" max="2" width="11.7109375" customWidth="true"/>
     <col min="3" max="3" width="12.7109375" customWidth="true"/>
-    <col min="4" max="4" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.7109375" customWidth="true"/>
-    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="12.7109375" customWidth="true"/>
     <col min="7" max="7" width="12.42578125" customWidth="true"/>
     <col min="8" max="8" width="11.7109375" customWidth="true"/>
   </cols>
@@ -130,7 +130,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G1" s="0" t="s">
         <v>12</v>
@@ -144,25 +144,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>9.7830800211364117</v>
+        <v>9.7908545571032519</v>
       </c>
       <c r="C2" s="0">
-        <v>0.99071521761240711</v>
+        <v>0.99057874721474515</v>
       </c>
       <c r="D2" s="0">
-        <v>0.11837250990914853</v>
+        <v>1.109134050882387</v>
       </c>
       <c r="E2" s="0">
-        <v>203.80329826047512</v>
+        <v>203.80348777036431</v>
       </c>
       <c r="F2" s="0">
-        <v>1.1090877275215556</v>
+        <v>0.11855530366764189</v>
       </c>
       <c r="G2" s="0">
-        <v>-24.124707942855245</v>
+        <v>-24.16198438114008</v>
       </c>
       <c r="H2" s="0">
-        <v>3.3702531716129629</v>
+        <v>3.370244958964272</v>
       </c>
     </row>
     <row r="3">
@@ -170,22 +170,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>12.17467095481317</v>
+        <v>12.174670968665104</v>
       </c>
       <c r="C3" s="0">
-        <v>0.97725920294453483</v>
+        <v>0.97725920197958516</v>
       </c>
       <c r="D3" s="0">
-        <v>0.13213001314674264</v>
+        <v>1.1093892160460761</v>
       </c>
       <c r="E3" s="0">
-        <v>167.52600459960277</v>
+        <v>167.52600323946646</v>
       </c>
       <c r="F3" s="0">
-        <v>1.1093892160912775</v>
+        <v>0.13213001406649094</v>
       </c>
       <c r="G3" s="0">
-        <v>-22.13521319016678</v>
+        <v>-22.13521316453371</v>
       </c>
       <c r="H3" s="0">
         <v>1.7850791804303163</v>
@@ -196,22 +196,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>14.853004568766471</v>
+        <v>14.85300457204618</v>
       </c>
       <c r="C4" s="0">
-        <v>0.94702099990040634</v>
+        <v>0.9470209995881016</v>
       </c>
       <c r="D4" s="0">
-        <v>0.16396348317747006</v>
+        <v>1.1109844830618696</v>
       </c>
       <c r="E4" s="0">
-        <v>151.29005863373965</v>
+        <v>151.29005830812935</v>
       </c>
       <c r="F4" s="0">
-        <v>1.1109844830778763</v>
+        <v>0.16396348347376799</v>
       </c>
       <c r="G4" s="0">
-        <v>-24.806044983711629</v>
+        <v>-24.80604497515036</v>
       </c>
       <c r="H4" s="0">
         <v>2.3111601242641355</v>
@@ -222,25 +222,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>15.794588653344469</v>
+        <v>15.794588652925945</v>
       </c>
       <c r="C5" s="0">
-        <v>0.92402303922238604</v>
+        <v>0.92402303925873885</v>
       </c>
       <c r="D5" s="0">
-        <v>0.19859162767062732</v>
+        <v>1.1226146668951553</v>
       </c>
       <c r="E5" s="0">
-        <v>155.71388199213632</v>
+        <v>155.71388203007447</v>
       </c>
       <c r="F5" s="0">
-        <v>1.1226146668930133</v>
+        <v>0.19859162763641647</v>
       </c>
       <c r="G5" s="0">
-        <v>-30.923473275730338</v>
+        <v>-30.923473277937433</v>
       </c>
       <c r="H5" s="0">
-        <v>2.4658007191273081</v>
+        <v>2.4658007191273112</v>
       </c>
     </row>
     <row r="6">
@@ -248,25 +248,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>13.771816002005963</v>
+        <v>13.771816001430597</v>
       </c>
       <c r="C6" s="0">
-        <v>0.95129568576599954</v>
+        <v>0.9512956857998629</v>
       </c>
       <c r="D6" s="0">
-        <v>0.15960913438855961</v>
+        <v>1.1109048201547236</v>
       </c>
       <c r="E6" s="0">
-        <v>164.69628950402301</v>
+        <v>164.69628953709582</v>
       </c>
       <c r="F6" s="0">
-        <v>1.110904820154559</v>
+        <v>0.15960913435486068</v>
       </c>
       <c r="G6" s="0">
-        <v>-26.28703220474473</v>
+        <v>-26.287032204473363</v>
       </c>
       <c r="H6" s="0">
-        <v>3.3545980071603143</v>
+        <v>3.3545980071603134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
p3 - p2 now is p3, issue solved for main cal, main data main val
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="216" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="229" uniqueCount="14">
   <si>
     <t>Q</t>
   </si>
@@ -106,9 +106,9 @@
     <col min="1" max="1" width="4.5703125" customWidth="true"/>
     <col min="2" max="2" width="11.7109375" customWidth="true"/>
     <col min="3" max="3" width="12.7109375" customWidth="true"/>
-    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.7109375" customWidth="true"/>
-    <col min="6" max="6" width="12.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
     <col min="7" max="7" width="12.42578125" customWidth="true"/>
     <col min="8" max="8" width="11.7109375" customWidth="true"/>
   </cols>
@@ -130,7 +130,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" s="0" t="s">
         <v>12</v>
@@ -144,25 +144,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>9.7908545571032519</v>
+        <v>9.7830800211364117</v>
       </c>
       <c r="C2" s="0">
-        <v>0.99057874721474515</v>
+        <v>0.99071521761240711</v>
       </c>
       <c r="D2" s="0">
-        <v>1.109134050882387</v>
+        <v>0.11837250990914853</v>
       </c>
       <c r="E2" s="0">
-        <v>203.80348777036431</v>
+        <v>203.80329826047512</v>
       </c>
       <c r="F2" s="0">
-        <v>0.11855530366764189</v>
+        <v>1.1090877275215556</v>
       </c>
       <c r="G2" s="0">
-        <v>-24.16198438114008</v>
+        <v>-24.124707942855245</v>
       </c>
       <c r="H2" s="0">
-        <v>3.370244958964272</v>
+        <v>3.3702531716129629</v>
       </c>
     </row>
     <row r="3">
@@ -170,22 +170,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>12.174670968665104</v>
+        <v>12.17467095481317</v>
       </c>
       <c r="C3" s="0">
-        <v>0.97725920197958516</v>
+        <v>0.97725920294453483</v>
       </c>
       <c r="D3" s="0">
-        <v>1.1093892160460761</v>
+        <v>0.13213001314674264</v>
       </c>
       <c r="E3" s="0">
-        <v>167.52600323946646</v>
+        <v>167.52600459960277</v>
       </c>
       <c r="F3" s="0">
-        <v>0.13213001406649094</v>
+        <v>1.1093892160912775</v>
       </c>
       <c r="G3" s="0">
-        <v>-22.13521316453371</v>
+        <v>-22.13521319016678</v>
       </c>
       <c r="H3" s="0">
         <v>1.7850791804303163</v>
@@ -196,22 +196,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>14.85300457204618</v>
+        <v>14.853004568766471</v>
       </c>
       <c r="C4" s="0">
-        <v>0.9470209995881016</v>
+        <v>0.94702099990040634</v>
       </c>
       <c r="D4" s="0">
-        <v>1.1109844830618696</v>
+        <v>0.16396348317747006</v>
       </c>
       <c r="E4" s="0">
-        <v>151.29005830812935</v>
+        <v>151.29005863373965</v>
       </c>
       <c r="F4" s="0">
-        <v>0.16396348347376799</v>
+        <v>1.1109844830778763</v>
       </c>
       <c r="G4" s="0">
-        <v>-24.80604497515036</v>
+        <v>-24.806044983711629</v>
       </c>
       <c r="H4" s="0">
         <v>2.3111601242641355</v>
@@ -222,25 +222,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>15.794588652925945</v>
+        <v>15.794588653344469</v>
       </c>
       <c r="C5" s="0">
-        <v>0.92402303925873885</v>
+        <v>0.92402303922238604</v>
       </c>
       <c r="D5" s="0">
-        <v>1.1226146668951553</v>
+        <v>0.19859162767062732</v>
       </c>
       <c r="E5" s="0">
-        <v>155.71388203007447</v>
+        <v>155.71388199213632</v>
       </c>
       <c r="F5" s="0">
-        <v>0.19859162763641647</v>
+        <v>1.1226146668930133</v>
       </c>
       <c r="G5" s="0">
-        <v>-30.923473277937433</v>
+        <v>-30.923473275730338</v>
       </c>
       <c r="H5" s="0">
-        <v>2.4658007191273112</v>
+        <v>2.4658007191273081</v>
       </c>
     </row>
     <row r="6">
@@ -248,25 +248,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>13.771816001430597</v>
+        <v>13.771816002005963</v>
       </c>
       <c r="C6" s="0">
-        <v>0.9512956857998629</v>
+        <v>0.95129568576599954</v>
       </c>
       <c r="D6" s="0">
-        <v>1.1109048201547236</v>
+        <v>0.15960913438855961</v>
       </c>
       <c r="E6" s="0">
-        <v>164.69628953709582</v>
+        <v>164.69628950402301</v>
       </c>
       <c r="F6" s="0">
-        <v>0.15960913435486068</v>
+        <v>1.110904820154559</v>
       </c>
       <c r="G6" s="0">
-        <v>-26.287032204473363</v>
+        <v>-26.28703220474473</v>
       </c>
       <c r="H6" s="0">
-        <v>3.3545980071603134</v>
+        <v>3.3545980071603143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
processin data to get fgures with axis font larger
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="106" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="122" uniqueCount="17">
   <si>
     <t>Q</t>
   </si>
@@ -112,17 +112,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" customWidth="true"/>
-    <col min="2" max="2" width="11.7109375" customWidth="true"/>
-    <col min="3" max="3" width="12.7109375" customWidth="true"/>
-    <col min="4" max="4" width="12.7109375" customWidth="true"/>
-    <col min="5" max="5" width="11.7109375" customWidth="true"/>
-    <col min="6" max="6" width="11.7109375" customWidth="true"/>
-    <col min="7" max="7" width="12.42578125" customWidth="true"/>
-    <col min="8" max="8" width="11.7109375" customWidth="true"/>
-    <col min="9" max="9" width="11.7109375" customWidth="true"/>
-    <col min="10" max="10" width="14" customWidth="true"/>
-    <col min="11" max="11" width="14.5703125" customWidth="true"/>
+    <col min="1" max="1" width="4.33203125" customWidth="true"/>
+    <col min="2" max="2" width="11.5546875" customWidth="true"/>
+    <col min="3" max="3" width="12.5546875" customWidth="true"/>
+    <col min="4" max="4" width="12.5546875" customWidth="true"/>
+    <col min="5" max="5" width="11.5546875" customWidth="true"/>
+    <col min="6" max="6" width="11.5546875" customWidth="true"/>
+    <col min="7" max="7" width="12.21875" customWidth="true"/>
+    <col min="8" max="8" width="11.5546875" customWidth="true"/>
+    <col min="9" max="9" width="11.5546875" customWidth="true"/>
+    <col min="10" max="10" width="13.109375" customWidth="true"/>
+    <col min="11" max="11" width="13.44140625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
cal and val scripts with update QAl results and figures with legend T_MFM for paper
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/nlfittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="122" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="138" uniqueCount="17">
   <si>
     <t>Q</t>
   </si>
@@ -112,17 +112,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.33203125" customWidth="true"/>
-    <col min="2" max="2" width="11.5546875" customWidth="true"/>
-    <col min="3" max="3" width="12.5546875" customWidth="true"/>
-    <col min="4" max="4" width="12.5546875" customWidth="true"/>
-    <col min="5" max="5" width="11.5546875" customWidth="true"/>
-    <col min="6" max="6" width="11.5546875" customWidth="true"/>
-    <col min="7" max="7" width="12.21875" customWidth="true"/>
-    <col min="8" max="8" width="11.5546875" customWidth="true"/>
-    <col min="9" max="9" width="11.5546875" customWidth="true"/>
-    <col min="10" max="10" width="13.109375" customWidth="true"/>
-    <col min="11" max="11" width="13.44140625" customWidth="true"/>
+    <col min="1" max="1" width="4.5703125" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+    <col min="7" max="7" width="12.42578125" customWidth="true"/>
+    <col min="8" max="8" width="11.7109375" customWidth="true"/>
+    <col min="9" max="9" width="11.7109375" customWidth="true"/>
+    <col min="10" max="10" width="14" customWidth="true"/>
+    <col min="11" max="11" width="14.5703125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>